<commit_message>
chore: auto update fair data
</commit_message>
<xml_diff>
--- a/build/events_master.xlsx
+++ b/build/events_master.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -736,7 +736,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -836,7 +836,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1036,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1736,7 +1736,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2236,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2736,7 +2736,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2836,7 +2836,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>2026-09-06T08:28:50+00:00</t>
+          <t>2026-09-07T09:06:20+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>